<commit_message>
corrected explicit CM implementation
</commit_message>
<xml_diff>
--- a/Results/analysis.xlsx
+++ b/Results/analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kadekola\github_codes\crossborder-CM\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90467BAA-8566-4266-8A7A-1F1F7014855C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1A07C79-6587-4C29-8F51-DAFC9567B74A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="1920" windowWidth="16440" windowHeight="28440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="analysis" sheetId="1" r:id="rId1"/>
@@ -156,7 +156,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -171,18 +171,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">

</xml_diff>

<commit_message>
last changes before exact projection method
</commit_message>
<xml_diff>
--- a/Results/analysis.xlsx
+++ b/Results/analysis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kadekola\github_codes\crossborder-CM\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1A07C79-6587-4C29-8F51-DAFC9567B74A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{582B95CB-D1EE-4CAB-9374-D8021318945D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,37 +36,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={3FA10FEE-C86A-4136-8FB8-090B68666114}</author>
-    <author>tc={0A1B3005-19DD-4398-AC20-DC7CA7B37746}</author>
-  </authors>
-  <commentList>
-    <comment ref="B12" authorId="0" shapeId="0" xr:uid="{3FA10FEE-C86A-4136-8FB8-090B68666114}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    CM price higher in zone C ~ 98,000.</t>
-      </text>
-    </comment>
-    <comment ref="B13" authorId="1" shapeId="0" xr:uid="{0A1B3005-19DD-4398-AC20-DC7CA7B37746}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    By setting the value of the internal line in zone A to a very high value
-Reply:
-    CM price convergence</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="30">
   <si>
     <t>Zone A</t>
   </si>
@@ -150,6 +121,12 @@
   </si>
   <si>
     <t>Explicit CM - FBMC</t>
+  </si>
+  <si>
+    <t>MEC</t>
+  </si>
+  <si>
+    <t>Without CM, maximum import</t>
   </si>
 </sst>
 </file>
@@ -3052,9 +3029,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>412012</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>178972</xdr:rowOff>
+      <xdr:colOff>408837</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>1172</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3098,7 +3075,7 @@
       <xdr:col>21</xdr:col>
       <xdr:colOff>231531</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>29734</xdr:rowOff>
+      <xdr:rowOff>26559</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3140,9 +3117,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>238641</xdr:colOff>
+      <xdr:colOff>235466</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>8016</xdr:rowOff>
+      <xdr:rowOff>11191</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3292,9 +3269,7 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Kamaldeen Adekola" id="{DEAC662C-4430-45A3-844D-88C8F1103BB6}" userId="S::kadekola@tudelft.nl::49d164b4-13c0-49ed-b3f1-423289268571" providerId="AD"/>
-</personList>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3558,20 +3533,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B12" dT="2025-04-07T13:32:43.14" personId="{DEAC662C-4430-45A3-844D-88C8F1103BB6}" id="{3FA10FEE-C86A-4136-8FB8-090B68666114}">
-    <text>CM price higher in zone C ~ 98,000.</text>
-  </threadedComment>
-  <threadedComment ref="B13" dT="2025-04-07T13:20:55.28" personId="{DEAC662C-4430-45A3-844D-88C8F1103BB6}" id="{0A1B3005-19DD-4398-AC20-DC7CA7B37746}">
-    <text>By setting the value of the internal line in zone A to a very high value</text>
-  </threadedComment>
-  <threadedComment ref="B13" dT="2025-04-07T13:32:08.72" personId="{DEAC662C-4430-45A3-844D-88C8F1103BB6}" id="{DA61E98C-BFC0-480A-BC6D-EE7B79D8704F}" parentId="{0A1B3005-19DD-4398-AC20-DC7CA7B37746}">
-    <text>CM price convergence</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S42"/>
@@ -4145,13 +4106,31 @@
         <v>76546.52</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" s="1"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" s="1"/>
     </row>
   </sheetData>
@@ -4162,7 +4141,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4C87616-DB5A-4675-84F3-F4854C3C9CFB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4C87616-DB5A-4675-84F3-F4854C3C9CFB}">
   <dimension ref="B1:F33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -4429,6 +4408,5 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
implemented exact projection for NetworkManager
</commit_message>
<xml_diff>
--- a/Results/analysis.xlsx
+++ b/Results/analysis.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kadekola\github_codes\crossborder-CM\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{582B95CB-D1EE-4CAB-9374-D8021318945D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AADF000-5499-438C-A539-5B1AC9B434E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="1920" windowWidth="16440" windowHeight="28440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="analysis" sheetId="1" r:id="rId1"/>
-    <sheet name="plot" sheetId="2" r:id="rId2"/>
+    <sheet name="NetworkManager_EP" sheetId="4" r:id="rId1"/>
+    <sheet name="analysis" sheetId="1" r:id="rId2"/>
+    <sheet name="plot" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,8 +37,35 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={8AF55A43-1AD8-4169-A1D2-9E54F7A217FB}</author>
+    <author>tc={6255527D-F628-4F1F-A30D-8CAA72ADDCFB}</author>
+  </authors>
+  <commentList>
+    <comment ref="H2" authorId="0" shapeId="0" xr:uid="{8AF55A43-1AD8-4169-A1D2-9E54F7A217FB}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Initial locally optimal error</t>
+      </text>
+    </comment>
+    <comment ref="K8" authorId="1" shapeId="0" xr:uid="{6255527D-F628-4F1F-A30D-8CAA72ADDCFB}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Creating energy on node 4</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="96">
   <si>
     <t>Zone A</t>
   </si>
@@ -127,13 +155,211 @@
   </si>
   <si>
     <t>Without CM, maximum import</t>
+  </si>
+  <si>
+    <t>julia&gt; value.(g_red)</t>
+  </si>
+  <si>
+    <t>2-dimensional DenseAxisArray{Float64,2,...} with index sets:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Dimension 1, 1:24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Dimension 2, 1:4</t>
+  </si>
+  <si>
+    <t>And data, a 24×4 Matrix{Float64}:</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1909.44   -1909.44    0.00565455  0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1998.94   -1998.94    0.00565455  0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1935.69   -1935.69    0.00565455  0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1943.96   -1943.96    0.00565455  0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ⋮</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1606.65   -1606.65    0.00783995  0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -241.958    241.958  -0.00353652  0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -262.073    262.073  -0.00450203  0.0</t>
+  </si>
+  <si>
+    <t>Without redispatch limit constraint</t>
+  </si>
+  <si>
+    <t>julia&gt; value.(flow)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1309.44   -3000.0  -1309.44   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1398.94   -3000.0  -1398.94   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1335.69   -3000.0  -1335.69   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1343.96   -3000.0  -1343.96   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1006.65   -3000.0  -1006.65   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -841.958  -3000.0    841.958  3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -862.073  -3000.0    862.073  3000.0</t>
+  </si>
+  <si>
+    <t>julia&gt; value.(ens)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -0.0  -0.0  -0.0  -0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ⋮</t>
+  </si>
+  <si>
+    <t>julia&gt; value.(ex)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Dimension 2, [(:A, :C), (:C, :B), (:B, :A)]</t>
+  </si>
+  <si>
+    <t>And data, a 24×3 Matrix{Float64}:</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0  -1309.44   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0  -1398.94   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0  -1335.69   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0  -1343.96   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     ⋮</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0  -1006.65   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0    841.958  3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0    862.073  3000.0</t>
+  </si>
+  <si>
+    <t>With redispatch limit constraint</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0  -647.32    3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0  -858.35    3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0  -775.235   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0  -765.717   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0    86.0348  3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0   849.158   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3000.0   865.914   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1247.32   -1247.32   -0.00261733  -13452.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1458.35   -1458.35   -0.00261738  -12924.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1375.23   -1375.23   -0.00261733  -12848.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1365.72   -1365.72   -0.00261733  -12821.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  513.965   -513.965  -3.64744e-9  -15744.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -249.158    249.158   0.047128    -15955.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -265.914    265.914   0.00864829  -15397.7</t>
+  </si>
+  <si>
+    <t>Non-convergence</t>
+  </si>
+  <si>
+    <t>Convergence at Iter=1035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  647.32    -3000.0  -647.32    3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  858.35    -3000.0  -858.35    3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  775.235   -3000.0  -775.235   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  765.717   -3000.0  -765.717   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  -86.0348  -3000.0    86.0348  3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -849.158   -3000.0   849.158   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -865.914   -3000.0   865.914   3000.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.49672e-25  -3.68861e-25  -5.59899e-22  -0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.08271e-25  -3.64539e-25  -6.26135e-23  -0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.7087e-25   -3.47728e-25  -7.36391e-23  -0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -5.02039e-25  -3.7745e-25   -8.74066e-23  -0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -4.75606e-25  -5.72739e-25  -1.61126e-9   -0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -3.18217e-25  -5.30265e-25  -4.79657e-24  -0.0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -148,6 +374,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -170,10 +409,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3269,7 +3509,9 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Kamaldeen Adekola" id="{6DC5C79D-D247-4DF2-A7CB-5B9F0353103B}" userId="S::kadekola@tudelft.nl::49d164b4-13c0-49ed-b3f1-423289268571" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3533,7 +3775,462 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="H2" dT="2025-05-26T12:43:07.67" personId="{6DC5C79D-D247-4DF2-A7CB-5B9F0353103B}" id="{8AF55A43-1AD8-4169-A1D2-9E54F7A217FB}">
+    <text>Initial locally optimal error</text>
+  </threadedComment>
+  <threadedComment ref="K8" dT="2025-05-26T12:41:12.86" personId="{6DC5C79D-D247-4DF2-A7CB-5B9F0353103B}" id="{6255527D-F628-4F1F-A30D-8CAA72ADDCFB}">
+    <text>Creating energy on node 4</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6DC44A-C910-475F-8505-F58C2C352113}">
+  <dimension ref="A1:K60"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>37</v>
+      </c>
+      <c r="H10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="H12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="H13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>31</v>
+      </c>
+      <c r="H19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="H20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>33</v>
+      </c>
+      <c r="H21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>34</v>
+      </c>
+      <c r="H22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>45</v>
+      </c>
+      <c r="H23" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="H24" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>47</v>
+      </c>
+      <c r="H25" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>48</v>
+      </c>
+      <c r="H26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>39</v>
+      </c>
+      <c r="H27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="H28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="H29" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>51</v>
+      </c>
+      <c r="H30" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="H34" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>32</v>
+      </c>
+      <c r="H35" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>33</v>
+      </c>
+      <c r="H36" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>34</v>
+      </c>
+      <c r="H37" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>53</v>
+      </c>
+      <c r="H38" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>53</v>
+      </c>
+      <c r="H39" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>53</v>
+      </c>
+      <c r="H40" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>53</v>
+      </c>
+      <c r="H41" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>54</v>
+      </c>
+      <c r="H42" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>53</v>
+      </c>
+      <c r="H43" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>53</v>
+      </c>
+      <c r="H44" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>55</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>31</v>
+      </c>
+      <c r="H49" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>32</v>
+      </c>
+      <c r="H50" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>56</v>
+      </c>
+      <c r="H51" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>57</v>
+      </c>
+      <c r="H52" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>58</v>
+      </c>
+      <c r="H53" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>59</v>
+      </c>
+      <c r="H54" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>60</v>
+      </c>
+      <c r="H55" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>61</v>
+      </c>
+      <c r="H56" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>62</v>
+      </c>
+      <c r="H57" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>63</v>
+      </c>
+      <c r="H58" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>64</v>
+      </c>
+      <c r="H59" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>65</v>
+      </c>
+      <c r="H60" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4140,7 +4837,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4C87616-DB5A-4675-84F3-F4854C3C9CFB}">
   <dimension ref="B1:F33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>